<commit_message>
Updated UI and Recorder
</commit_message>
<xml_diff>
--- a/test-data/Templates/DEV/R1 - RDS - create traded material(s).xlsx
+++ b/test-data/Templates/DEV/R1 - RDS - create traded material(s).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tejavathidoddapaneni/Maextro_AutomationApp/test-data/Templates/DEV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E61976FA-BE9A-EB43-9F5B-93EF739F97F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F9B494-AE5C-B442-B42D-8FC96DB5CB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{9B722DE1-D4F2-8E4B-A1FC-B7FBF3A04462}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{9B722DE1-D4F2-8E4B-A1FC-B7FBF3A04462}"/>
   </bookViews>
   <sheets>
     <sheet name="MXT_HDR" sheetId="1" r:id="rId1"/>
@@ -110,9 +110,6 @@
     <t>Request Number</t>
   </si>
   <si>
-    <t>Save</t>
-  </si>
-  <si>
     <t>Material</t>
   </si>
   <si>
@@ -626,9 +623,6 @@
     <t>Rejecting To</t>
   </si>
   <si>
-    <t>Approve</t>
-  </si>
-  <si>
     <t>R1 - RDS - create traded material(s)</t>
   </si>
   <si>
@@ -645,6 +639,12 @@
   </si>
   <si>
     <t xml:space="preserve">Add Records - </t>
+  </si>
+  <si>
+    <t>Skip</t>
+  </si>
+  <si>
+    <t>Reject -&gt; Approve</t>
   </si>
 </sst>
 </file>
@@ -1101,16 +1101,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -1119,7 +1119,7 @@
         <v>9</v>
       </c>
       <c r="H2">
-        <v>39444</v>
+        <v>23033</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1136,7 +1136,7 @@
         <v>14</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1149,10 +1149,10 @@
         <v>11</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1163,10 +1163,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>199</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -1177,10 +1180,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1191,10 +1194,10 @@
         <v>12</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -1205,10 +1208,10 @@
         <v>12</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -1219,10 +1222,10 @@
         <v>12</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1233,10 +1236,10 @@
         <v>12</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -1247,10 +1250,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1261,13 +1264,13 @@
         <v>15</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D14" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E14">
-        <v>400</v>
+        <v>700</v>
       </c>
     </row>
     <row r="23" spans="7:7" x14ac:dyDescent="0.2">
@@ -1275,9 +1278,6 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D6:D11 D13:D14 D12" xr:uid="{58227CB0-C6D9-A247-A15C-D0FCE8718EAF}">
-      <formula1>"Save,Skip,Approve,Reject -&gt; Approve"</formula1>
-    </dataValidation>
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{480D1B17-2E92-9240-8BCE-1DA3147CCDB2}">
       <formula1>"Create New Material,Create Sales Pricing,New Sales Condition record,Create Purchase Order,Create Purchase requisition,Create Production Version,Habasit training"</formula1>
     </dataValidation>
@@ -1286,6 +1286,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{867B6D3F-F6EA-6D45-89A3-70B9CE3A4229}">
       <formula1>"Low,Medium,High"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D6:D14" xr:uid="{1CFA1481-36A9-4D40-8774-9EBF4F3DD350}">
+      <formula1>"Save,Skip,Approve,Reject -&gt; Approve,Skip -&gt; Save ,Skip -&gt; Approve"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1299,16 +1302,16 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
@@ -1316,43 +1319,43 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
@@ -1362,16 +1365,16 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -1379,22 +1382,22 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -1404,16 +1407,16 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -1421,16 +1424,16 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -1440,16 +1443,16 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
@@ -1457,13 +1460,13 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -1473,16 +1476,16 @@
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
@@ -1490,40 +1493,40 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="K18" s="2" t="s">
+      <c r="L18" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="M18" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
@@ -1533,16 +1536,16 @@
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.2">
@@ -1550,31 +1553,31 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F22" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G22" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="H22" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="J22" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.2">
@@ -1584,16 +1587,16 @@
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
@@ -1601,10 +1604,10 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>17</v>
@@ -1613,55 +1616,55 @@
         <v>18</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H26" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="L26" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="L26" s="1" t="s">
+      <c r="M26" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="M26" s="1" t="s">
+      <c r="N26" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="N26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="O26" s="1" t="s">
+      <c r="P26" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="P26" s="1" t="s">
+      <c r="Q26" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Q26" s="1" t="s">
+      <c r="R26" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="R26" s="1" t="s">
+      <c r="S26" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="S26" s="1" t="s">
+      <c r="T26" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="T26" s="1" t="s">
+      <c r="U26" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="U26" s="1" t="s">
+      <c r="V26" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="V26" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
@@ -1673,16 +1676,16 @@
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
@@ -1690,22 +1693,22 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>17</v>
@@ -1723,16 +1726,16 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
@@ -1740,25 +1743,25 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E34" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="G34" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H34" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
@@ -1768,16 +1771,16 @@
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.2">
@@ -1785,13 +1788,13 @@
         <v>19</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
@@ -1801,16 +1804,16 @@
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.2">
@@ -1818,55 +1821,55 @@
         <v>19</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F42" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="H42" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I42" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="H42" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I42" s="1" t="s">
+      <c r="J42" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="J42" s="1" t="s">
+      <c r="K42" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="K42" s="1" t="s">
+      <c r="L42" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="M42" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="L42" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="M42" s="1" t="s">
+      <c r="N42" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="N42" s="1" t="s">
+      <c r="O42" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="O42" s="1" t="s">
+      <c r="P42" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="P42" s="1" t="s">
+      <c r="Q42" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="Q42" s="1" t="s">
+      <c r="R42" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="R42" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.2">
@@ -1877,16 +1880,16 @@
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.2">
@@ -1894,16 +1897,16 @@
         <v>19</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.2">
@@ -1913,16 +1916,16 @@
     </row>
     <row r="49" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" spans="1:30" x14ac:dyDescent="0.2">
@@ -1930,22 +1933,22 @@
         <v>19</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D50" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="F50" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="G50" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:30" x14ac:dyDescent="0.2">
@@ -1955,16 +1958,16 @@
     </row>
     <row r="53" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
@@ -1974,91 +1977,91 @@
         <v>19</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N54" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="O54" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="P54" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q54" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="R54" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="S54" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="T54" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="U54" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="V54" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="W54" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="X54" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="Y54" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="Z54" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA54" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB54" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="N54" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="P54" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q54" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="R54" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="S54" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="T54" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="U54" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="V54" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="W54" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="X54" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y54" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="Z54" s="1" t="s">
+      <c r="AC54" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="AA54" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AB54" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AC54" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="AD54" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="55" spans="1:30" x14ac:dyDescent="0.2">
@@ -2070,16 +2073,16 @@
     </row>
     <row r="57" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
@@ -2090,40 +2093,40 @@
         <v>19</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F58" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H58" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="G58" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H58" s="1" t="s">
+      <c r="I58" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="I58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J58" s="1" t="s">
+      <c r="K58" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K58" s="1" t="s">
+      <c r="L58" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="L58" s="1" t="s">
+      <c r="M58" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="M58" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.2">
@@ -2133,16 +2136,16 @@
     </row>
     <row r="61" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="62" spans="1:30" x14ac:dyDescent="0.2">
@@ -2150,28 +2153,28 @@
         <v>19</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F62" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="H62" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="63" spans="1:30" x14ac:dyDescent="0.2">
@@ -2181,16 +2184,16 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
@@ -2198,37 +2201,37 @@
         <v>19</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G66" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="F66" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="H66" s="1" t="s">
+      <c r="I66" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I66" s="1" t="s">
+      <c r="J66" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="J66" s="1" t="s">
+      <c r="K66" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="K66" s="1" t="s">
+      <c r="L66" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="L66" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
@@ -2238,16 +2241,16 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
@@ -2255,34 +2258,34 @@
         <v>19</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="G70" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="H70" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="H70" s="1" t="s">
+      <c r="I70" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="I70" s="1" t="s">
+      <c r="J70" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J70" s="1" t="s">
+      <c r="K70" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
@@ -2321,16 +2324,16 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
@@ -2338,43 +2341,43 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
@@ -2382,30 +2385,30 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
         <v>41</v>
-      </c>
-      <c r="E3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -2413,16 +2416,16 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -2438,16 +2441,16 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -2455,7 +2458,7 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>18</v>
@@ -2476,16 +2479,16 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
@@ -2493,22 +2496,22 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -2520,16 +2523,16 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
@@ -2537,13 +2540,13 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -2558,16 +2561,16 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -2575,22 +2578,22 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
@@ -2600,16 +2603,16 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
@@ -2617,40 +2620,40 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="E26" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="H26" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="K26" s="2" t="s">
+      <c r="L26" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="M26" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
@@ -2658,21 +2661,21 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
@@ -2680,16 +2683,16 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
@@ -2699,16 +2702,16 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -2716,13 +2719,13 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -2759,16 +2762,16 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
@@ -2776,43 +2779,43 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -2822,16 +2825,16 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -2839,13 +2842,13 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -2894,16 +2897,16 @@
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.2">
@@ -2911,43 +2914,43 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.2">
@@ -2957,16 +2960,16 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2">
@@ -2974,22 +2977,22 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>17</v>
@@ -3010,16 +3013,16 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.2">
@@ -3027,10 +3030,10 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>17</v>
@@ -3039,55 +3042,55 @@
         <v>18</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="K10" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="L10" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="M10" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="N10" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="N10" s="1" t="s">
+      <c r="O10" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="O10" s="1" t="s">
+      <c r="P10" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="1" t="s">
+      <c r="Q10" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Q10" s="1" t="s">
+      <c r="R10" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="R10" s="1" t="s">
+      <c r="S10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="T10" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="T10" s="1" t="s">
+      <c r="U10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="U10" s="1" t="s">
+      <c r="V10" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
@@ -3097,21 +3100,21 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="O11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.2">
@@ -3119,31 +3122,31 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F14" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
@@ -3151,21 +3154,21 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -3173,25 +3176,25 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -3201,16 +3204,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -3218,13 +3221,13 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -3266,16 +3269,16 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
@@ -3283,55 +3286,55 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -3339,21 +3342,21 @@
         <v>1</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -3361,16 +3364,16 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
@@ -3380,16 +3383,16 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
@@ -3397,22 +3400,22 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="G10" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -3460,16 +3463,16 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -3479,91 +3482,91 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="AA2" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="AD2" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.2">
@@ -3571,19 +3574,19 @@
         <v>1</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O3">
         <v>10</v>
@@ -3594,16 +3597,16 @@
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -3614,40 +3617,40 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.2">
@@ -3680,16 +3683,16 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -3697,28 +3700,28 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -3751,16 +3754,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
@@ -3768,34 +3771,34 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -3828,16 +3831,16 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -3845,37 +3848,37 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -3886,13 +3889,13 @@
         <v>3100</v>
       </c>
       <c r="H3" t="s">
+        <v>186</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="s">
         <v>187</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="L3" t="s">
-        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>